<commit_message>
P1: requirements, architecture, localization docs, prompts and agent instructions
Phase P1 documentation under Approval B:
- docs/: product, design, architecture (+18 ADRs), localization, api (proposed),
  testing, security, project-management and release docs with Mermaid flow,
  sequence and state diagrams
- prompts/00-21 and per-ticket prompts for the 26 P2 tickets
- CLAUDE.md and .github/copilot-instructions.md (same rules), PR template,
  CODEOWNERS, .gitattributes, README
- Backlog workbook: decisions D1-D15, risks R-21-R-24, new tickets LS-009 and
  LS-039, NFR-13-17, TC-059-061, 7-feature module mapping, P1 ticket statuses

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AyK9D11zqoszoFoKLWcJTJ
</commit_message>
<xml_diff>
--- a/docs/project-management/LittleStory_Jira_Backlog.xlsx
+++ b/docs/project-management/LittleStory_Jira_Backlog.xlsx
@@ -27,15 +27,15 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="18" state="hidden" r:id="rId18"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog'!$A$1:$AL$83</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog'!$A$1:$AL$85</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Epics'!$A$1:$I$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Screens'!$A$1:$S$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Design System'!$A$4:$E$66</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Requirements'!$A$1:$J$38</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Test Cases'!$A$1:$P$59</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Dependencies'!$A$1:$M$83</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'ADRs'!$A$1:$K$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Risks &amp; Questions'!$A$1:$K$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Requirements'!$A$1:$J$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Test Cases'!$A$1:$P$62</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Dependencies'!$A$1:$M$94</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'ADRs'!$A$1:$K$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Risks &amp; Questions'!$A$1:$K$25</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'Git-PR-CI'!$A$1:$P$83</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'Translations'!$A$1:$I$296</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'Prompt Library'!$A$1:$F$25</definedName>
@@ -760,6 +760,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -785,6 +788,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -810,6 +816,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -835,6 +844,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -860,6 +872,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -885,6 +900,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -910,6 +928,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -935,6 +956,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -960,6 +984,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -985,6 +1012,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1010,6 +1040,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1035,6 +1068,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1060,6 +1096,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1085,6 +1124,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1110,6 +1152,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1135,6 +1180,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1160,6 +1208,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1185,6 +1236,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1210,6 +1264,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1235,6 +1292,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1265,6 +1325,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1290,6 +1353,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1315,6 +1381,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1340,6 +1409,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1365,6 +1437,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1390,6 +1465,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1415,6 +1493,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1440,6 +1521,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1465,6 +1549,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1490,6 +1577,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1515,6 +1605,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1540,6 +1633,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1565,6 +1661,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1590,6 +1689,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1615,6 +1717,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1640,6 +1745,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1665,6 +1773,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1690,6 +1801,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1715,6 +1829,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1740,6 +1857,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1765,6 +1885,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1790,6 +1913,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2284,7 +2410,7 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>P0 Discovery – design inventory done from design pack (LS-002); repository discovery (LS-001) pending.</t>
+          <t>P1 Requirements &amp; planning — Approval B granted 29 Oct 2026; docs, prompts, CLAUDE.md and copilot instructions drafted on claude/project-thread-veobz7, awaiting owner review. P0 discovery (LS-001, LS-002) done.</t>
         </is>
       </c>
     </row>
@@ -2296,7 +2422,7 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Old 'LittleKatha' brand in designs · 7 design languages vs EN/KN · fonts lack Kannada glyphs · missing designs (splash, language prefs, privacy, help) · contrast &amp; touch targets · Kannada reviewer availability. See 'Risks &amp; Questions'.</t>
+          <t>Old 'LittleKatha' brand in designs · 7 design languages vs EN/KN · fonts lack Kannada glyphs · missing designs (splash, language prefs, privacy, help) · contrast &amp; touch targets · Kannada reviewer availability. See 'Risks &amp; Questions' · cloud workspace cannot build Android (R-21) · default branch misconfigured (R-22).</t>
         </is>
       </c>
     </row>
@@ -2467,7 +2593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J38"/>
+  <dimension ref="A1:J43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2582,7 +2708,7 @@
       </c>
       <c r="J2" s="4" t="inlineStr">
         <is>
-          <t>Proposed – awaiting Approval B</t>
+          <t>Proposed – awaiting owner review</t>
         </is>
       </c>
     </row>
@@ -2634,7 +2760,7 @@
       </c>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>Proposed – awaiting Approval B</t>
+          <t>Proposed – awaiting owner review</t>
         </is>
       </c>
     </row>
@@ -2686,7 +2812,7 @@
       </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
-          <t>Proposed – awaiting Approval B</t>
+          <t>Proposed – awaiting owner review</t>
         </is>
       </c>
     </row>
@@ -2738,7 +2864,7 @@
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>Proposed – awaiting Approval B</t>
+          <t>Proposed – awaiting owner review</t>
         </is>
       </c>
     </row>
@@ -2790,7 +2916,7 @@
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t>Proposed – awaiting Approval B</t>
+          <t>Proposed – awaiting owner review</t>
         </is>
       </c>
     </row>
@@ -2842,7 +2968,7 @@
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>Proposed – awaiting Approval B</t>
+          <t>Proposed – awaiting owner review</t>
         </is>
       </c>
     </row>
@@ -2894,7 +3020,7 @@
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
-          <t>Proposed – awaiting Approval B</t>
+          <t>Proposed – awaiting owner review</t>
         </is>
       </c>
     </row>
@@ -2941,12 +3067,12 @@
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>TC-019, TC-020, TC-021, TC-022</t>
+          <t>TC-019, TC-020, TC-021, TC-022, TC-061</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>Proposed – awaiting Approval B</t>
+          <t>Proposed – awaiting owner review</t>
         </is>
       </c>
     </row>
@@ -2998,7 +3124,7 @@
       </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
-          <t>Proposed – awaiting Approval B</t>
+          <t>Proposed – awaiting owner review</t>
         </is>
       </c>
     </row>
@@ -3050,7 +3176,7 @@
       </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
-          <t>Proposed – awaiting Approval B</t>
+          <t>Proposed – awaiting owner review</t>
         </is>
       </c>
     </row>
@@ -3102,7 +3228,7 @@
       </c>
       <c r="J12" s="4" t="inlineStr">
         <is>
-          <t>Proposed – awaiting Approval B</t>
+          <t>Proposed – awaiting owner review</t>
         </is>
       </c>
     </row>
@@ -3154,7 +3280,7 @@
       </c>
       <c r="J13" s="4" t="inlineStr">
         <is>
-          <t>Proposed – awaiting Approval B</t>
+          <t>Proposed – awaiting owner review</t>
         </is>
       </c>
     </row>
@@ -3206,7 +3332,7 @@
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
-          <t>Proposed – awaiting Approval B</t>
+          <t>Proposed – awaiting owner review</t>
         </is>
       </c>
     </row>
@@ -3258,7 +3384,7 @@
       </c>
       <c r="J15" s="4" t="inlineStr">
         <is>
-          <t>Proposed – awaiting Approval B</t>
+          <t>Proposed – awaiting owner review</t>
         </is>
       </c>
     </row>
@@ -3310,7 +3436,7 @@
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
-          <t>Proposed – awaiting Approval B</t>
+          <t>Proposed – awaiting owner review</t>
         </is>
       </c>
     </row>
@@ -3362,7 +3488,7 @@
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
-          <t>Proposed – awaiting Approval B</t>
+          <t>Proposed – awaiting owner review</t>
         </is>
       </c>
     </row>
@@ -3414,7 +3540,7 @@
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
-          <t>Proposed – awaiting Approval B</t>
+          <t>Proposed – awaiting owner review</t>
         </is>
       </c>
     </row>
@@ -3466,7 +3592,7 @@
       </c>
       <c r="J19" s="4" t="inlineStr">
         <is>
-          <t>Proposed – awaiting Approval B</t>
+          <t>Proposed – awaiting owner review</t>
         </is>
       </c>
     </row>
@@ -3518,7 +3644,7 @@
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>Proposed – awaiting Approval B</t>
+          <t>Proposed – awaiting owner review</t>
         </is>
       </c>
     </row>
@@ -3570,7 +3696,7 @@
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>Proposed – awaiting Approval B</t>
+          <t>Proposed – awaiting owner review</t>
         </is>
       </c>
     </row>
@@ -3617,12 +3743,12 @@
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>TC-023</t>
+          <t>TC-023, TC-060</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
-          <t>Proposed – awaiting Approval B</t>
+          <t>Proposed – awaiting owner review</t>
         </is>
       </c>
     </row>
@@ -3674,7 +3800,7 @@
       </c>
       <c r="J23" s="4" t="inlineStr">
         <is>
-          <t>Proposed – awaiting Approval B</t>
+          <t>Proposed – awaiting owner review</t>
         </is>
       </c>
     </row>
@@ -3726,7 +3852,7 @@
       </c>
       <c r="J24" s="4" t="inlineStr">
         <is>
-          <t>Proposed – awaiting Approval B</t>
+          <t>Proposed – awaiting owner review</t>
         </is>
       </c>
     </row>
@@ -3778,7 +3904,7 @@
       </c>
       <c r="J25" s="4" t="inlineStr">
         <is>
-          <t>Proposed – awaiting Approval B</t>
+          <t>Proposed – awaiting owner review</t>
         </is>
       </c>
     </row>
@@ -3830,7 +3956,7 @@
       </c>
       <c r="J26" s="4" t="inlineStr">
         <is>
-          <t>Proposed – awaiting Approval B</t>
+          <t>Proposed – awaiting owner review</t>
         </is>
       </c>
     </row>
@@ -3882,7 +4008,7 @@
       </c>
       <c r="J27" s="4" t="inlineStr">
         <is>
-          <t>Proposed – awaiting Approval B</t>
+          <t>Proposed – awaiting owner review</t>
         </is>
       </c>
     </row>
@@ -3934,7 +4060,7 @@
       </c>
       <c r="J28" s="4" t="inlineStr">
         <is>
-          <t>Proposed – awaiting Approval B</t>
+          <t>Proposed – awaiting owner review</t>
         </is>
       </c>
     </row>
@@ -3981,12 +4107,12 @@
       </c>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>TC-052</t>
+          <t>TC-052, TC-059</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
         <is>
-          <t>Proposed – awaiting Approval B</t>
+          <t>Proposed – awaiting owner review</t>
         </is>
       </c>
     </row>
@@ -4038,7 +4164,7 @@
       </c>
       <c r="J30" s="4" t="inlineStr">
         <is>
-          <t>Proposed – awaiting Approval B</t>
+          <t>Proposed – awaiting owner review</t>
         </is>
       </c>
     </row>
@@ -4090,7 +4216,7 @@
       </c>
       <c r="J31" s="4" t="inlineStr">
         <is>
-          <t>Proposed – awaiting Approval B</t>
+          <t>Proposed – awaiting owner review</t>
         </is>
       </c>
     </row>
@@ -4142,7 +4268,7 @@
       </c>
       <c r="J32" s="4" t="inlineStr">
         <is>
-          <t>Proposed – awaiting Approval B</t>
+          <t>Proposed – awaiting owner review</t>
         </is>
       </c>
     </row>
@@ -4194,7 +4320,7 @@
       </c>
       <c r="J33" s="4" t="inlineStr">
         <is>
-          <t>Proposed – awaiting Approval B</t>
+          <t>Proposed – awaiting owner review</t>
         </is>
       </c>
     </row>
@@ -4246,7 +4372,7 @@
       </c>
       <c r="J34" s="4" t="inlineStr">
         <is>
-          <t>Proposed – awaiting Approval B</t>
+          <t>Proposed – awaiting owner review</t>
         </is>
       </c>
     </row>
@@ -4298,7 +4424,7 @@
       </c>
       <c r="J35" s="4" t="inlineStr">
         <is>
-          <t>Proposed – awaiting Approval B</t>
+          <t>Proposed – awaiting owner review</t>
         </is>
       </c>
     </row>
@@ -4350,7 +4476,7 @@
       </c>
       <c r="J36" s="4" t="inlineStr">
         <is>
-          <t>Proposed – awaiting Approval B</t>
+          <t>Proposed – awaiting owner review</t>
         </is>
       </c>
     </row>
@@ -4402,7 +4528,7 @@
       </c>
       <c r="J37" s="4" t="inlineStr">
         <is>
-          <t>Proposed – awaiting Approval B</t>
+          <t>Proposed – awaiting owner review</t>
         </is>
       </c>
     </row>
@@ -4454,12 +4580,272 @@
       </c>
       <c r="J38" s="4" t="inlineStr">
         <is>
-          <t>Proposed – awaiting Approval B</t>
+          <t>Proposed – awaiting owner review</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="31" customHeight="1">
+      <c r="A39" s="17" t="inlineStr">
+        <is>
+          <t>NFR-13</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>Non-functional</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>Locale-aware formatting</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>Numbers, dates, times, durations, weekdays and currency formatted with locale-aware APIs; no concatenation</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>Brief §4.4 rule 12, §8.7 (NEW, proposed)</t>
+        </is>
+      </c>
+      <c r="G39" s="4" t="inlineStr">
+        <is>
+          <t>SCR-11a, SCR-15, SCR-16, SCR-17</t>
+        </is>
+      </c>
+      <c r="H39" s="4" t="inlineStr">
+        <is>
+          <t>LS-040, LS-092, LS-101, LS-111, LS-113</t>
+        </is>
+      </c>
+      <c r="I39" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J39" s="4" t="inlineStr">
+        <is>
+          <t>Proposed – awaiting owner review</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="31" customHeight="1">
+      <c r="A40" s="17" t="inlineStr">
+        <is>
+          <t>NFR-14</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>Non-functional</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>RTL and text-expansion readiness</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>supportsRtl, start/end only, flexible text containers; en-XA and ar-XB pseudo-locales render without clipping</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t>Brief §4.4 rules 10, 11, 18 (NEW, proposed)</t>
+        </is>
+      </c>
+      <c r="G40" s="4" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="H40" s="4" t="inlineStr">
+        <is>
+          <t>LS-013, LS-016, LS-019, LS-042</t>
+        </is>
+      </c>
+      <c r="I40" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J40" s="4" t="inlineStr">
+        <is>
+          <t>Proposed – awaiting owner review</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="31" customHeight="1">
+      <c r="A41" s="17" t="inlineStr">
+        <is>
+          <t>NFR-15</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>Non-functional</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>Configurability and How to change X</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>Every configurable value has one documented home; changing wording, colour, limit or mock story edits one file</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>Brief §4.5, §8.8 (NEW, proposed)</t>
+        </is>
+      </c>
+      <c r="G41" s="4" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="H41" s="4" t="inlineStr">
+        <is>
+          <t>LS-033, LS-125, LS-150</t>
+        </is>
+      </c>
+      <c r="I41" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J41" s="4" t="inlineStr">
+        <is>
+          <t>Proposed – awaiting owner review</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="31" customHeight="1">
+      <c r="A42" s="17" t="inlineStr">
+        <is>
+          <t>NFR-16</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>Non-functional</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>Compatibility and device matrix</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>Supported Android versions (minSdk per ADR-016), screen sizes and test devices documented and tested</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="inlineStr">
+        <is>
+          <t>Brief §8.6 (NEW, proposed)</t>
+        </is>
+      </c>
+      <c r="G42" s="4" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="H42" s="4" t="inlineStr">
+        <is>
+          <t>LS-030, LS-132</t>
+        </is>
+      </c>
+      <c r="I42" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J42" s="4" t="inlineStr">
+        <is>
+          <t>Proposed – awaiting owner review</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="31" customHeight="1">
+      <c r="A43" s="17" t="inlineStr">
+        <is>
+          <t>NFR-17</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>Non-functional</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>Build verifiability</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>Every PR carries build, test and lint evidence from CI or a documented local run; no unverified claims</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr">
+        <is>
+          <t>P0 finding R-21 (NEW, proposed)</t>
+        </is>
+      </c>
+      <c r="G43" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H43" s="4" t="inlineStr">
+        <is>
+          <t>LS-039, LS-130, LS-030</t>
+        </is>
+      </c>
+      <c r="I43" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J43" s="4" t="inlineStr">
+        <is>
+          <t>Proposed – awaiting owner review</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J38"/>
+  <autoFilter ref="A1:J43"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4471,7 +4857,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P59"/>
+  <dimension ref="A1:P62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -8866,8 +9252,230 @@
       <c r="O59" s="4" t="inlineStr"/>
       <c r="P59" s="4" t="inlineStr"/>
     </row>
+    <row r="60" ht="18" customHeight="1">
+      <c r="A60" s="17" t="inlineStr">
+        <is>
+          <t>TC-059</t>
+        </is>
+      </c>
+      <c r="B60" s="4" t="inlineStr">
+        <is>
+          <t>LS-041</t>
+        </is>
+      </c>
+      <c r="C60" s="4" t="inlineStr">
+        <is>
+          <t>NFR-03</t>
+        </is>
+      </c>
+      <c r="D60" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E60" s="4" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="F60" s="4" t="inlineStr">
+        <is>
+          <t>Registry matches locales_config.xml</t>
+        </is>
+      </c>
+      <c r="G60" s="4" t="inlineStr">
+        <is>
+          <t>Registry and locales_config.xml exist</t>
+        </is>
+      </c>
+      <c r="H60" s="4" t="inlineStr">
+        <is>
+          <t>Run unit test comparing SupportedLanguage entries with locales_config.xml</t>
+        </is>
+      </c>
+      <c r="I60" s="4" t="inlineStr">
+        <is>
+          <t>Same locale set; test fails on mismatch</t>
+        </is>
+      </c>
+      <c r="J60" s="4" t="inlineStr">
+        <is>
+          <t>Localization</t>
+        </is>
+      </c>
+      <c r="K60" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L60" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M60" s="4" t="inlineStr">
+        <is>
+          <t>Registry + XML</t>
+        </is>
+      </c>
+      <c r="N60" s="4" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="O60" s="4" t="n"/>
+      <c r="P60" s="4" t="n"/>
+    </row>
+    <row r="61" ht="18" customHeight="1">
+      <c r="A61" s="17" t="inlineStr">
+        <is>
+          <t>TC-060</t>
+        </is>
+      </c>
+      <c r="B61" s="4" t="inlineStr">
+        <is>
+          <t>LS-036</t>
+        </is>
+      </c>
+      <c r="C61" s="4" t="inlineStr">
+        <is>
+          <t>FR-21</t>
+        </is>
+      </c>
+      <c r="D61" s="4" t="inlineStr">
+        <is>
+          <t>SCR-04a, SCR-06</t>
+        </is>
+      </c>
+      <c r="E61" s="4" t="inlineStr">
+        <is>
+          <t>en, kn</t>
+        </is>
+      </c>
+      <c r="F61" s="4" t="inlineStr">
+        <is>
+          <t>Mock content parity per story ID</t>
+        </is>
+      </c>
+      <c r="G61" s="4" t="inlineStr">
+        <is>
+          <t>stories_en.json and stories_kn.json present</t>
+        </is>
+      </c>
+      <c r="H61" s="4" t="inlineStr">
+        <is>
+          <t>Run parity check over all story IDs</t>
+        </is>
+      </c>
+      <c r="I61" s="4" t="inlineStr">
+        <is>
+          <t>Every ID exists in both files or is listed as expected English fallback (story_lanterns_jaipur)</t>
+        </is>
+      </c>
+      <c r="J61" s="4" t="inlineStr">
+        <is>
+          <t>Localization</t>
+        </is>
+      </c>
+      <c r="K61" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L61" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M61" s="4" t="inlineStr">
+        <is>
+          <t>docs/testing/test-data.md seed set</t>
+        </is>
+      </c>
+      <c r="N61" s="4" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="O61" s="4" t="n"/>
+      <c r="P61" s="4" t="n"/>
+    </row>
+    <row r="62" ht="18" customHeight="1">
+      <c r="A62" s="17" t="inlineStr">
+        <is>
+          <t>TC-061</t>
+        </is>
+      </c>
+      <c r="B62" s="4" t="inlineStr">
+        <is>
+          <t>LS-080</t>
+        </is>
+      </c>
+      <c r="C62" s="4" t="inlineStr">
+        <is>
+          <t>FR-08</t>
+        </is>
+      </c>
+      <c r="D62" s="4" t="inlineStr">
+        <is>
+          <t>SCR-07</t>
+        </is>
+      </c>
+      <c r="E62" s="4" t="inlineStr">
+        <is>
+          <t>kn</t>
+        </is>
+      </c>
+      <c r="F62" s="4" t="inlineStr">
+        <is>
+          <t>Kannada keyboard input in Create</t>
+        </is>
+      </c>
+      <c r="G62" s="4" t="inlineStr">
+        <is>
+          <t>App in Kannada, Kannada IME installed</t>
+        </is>
+      </c>
+      <c r="H62" s="4" t="inlineStr">
+        <is>
+          <t>Type a Kannada sentence in What happened today; submit</t>
+        </is>
+      </c>
+      <c r="I62" s="4" t="inlineStr">
+        <is>
+          <t>Text accepted, counter counts characters correctly, no clipping</t>
+        </is>
+      </c>
+      <c r="J62" s="4" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="K62" s="4" t="inlineStr">
+        <is>
+          <t>Partly</t>
+        </is>
+      </c>
+      <c r="L62" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="M62" s="4" t="inlineStr">
+        <is>
+          <t>Kannada sample sentence</t>
+        </is>
+      </c>
+      <c r="N62" s="4" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="O62" s="4" t="n"/>
+      <c r="P62" s="4" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P59"/>
+  <autoFilter ref="A1:P62"/>
   <conditionalFormatting sqref="N2:N109">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="9">
       <formula>"Pass"</formula>
@@ -8895,7 +9503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M92"/>
+  <dimension ref="A1:M94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -10266,7 +10874,7 @@
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>LS-001, LS-008</t>
+          <t>LS-001, LS-008, LS-009, LS-039</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
@@ -14607,8 +15215,142 @@
       <c r="G92" s="62" t="n"/>
       <c r="H92" s="61" t="n"/>
     </row>
+    <row r="93">
+      <c r="A93" s="17" t="inlineStr">
+        <is>
+          <t>LS-009</t>
+        </is>
+      </c>
+      <c r="B93" s="61" t="inlineStr">
+        <is>
+          <t>Repository hygiene: default branch main, development branch</t>
+        </is>
+      </c>
+      <c r="C93" s="4" t="inlineStr">
+        <is>
+          <t>LS-001</t>
+        </is>
+      </c>
+      <c r="D93" s="62" t="inlineStr">
+        <is>
+          <t>LS-001</t>
+        </is>
+      </c>
+      <c r="E93" s="62" t="inlineStr">
+        <is>
+          <t>LS-030, LS-131</t>
+        </is>
+      </c>
+      <c r="F93" s="62" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G93" s="62" t="inlineStr">
+        <is>
+          <t>GitHub settings</t>
+        </is>
+      </c>
+      <c r="H93" s="61" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>P1 exit</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>Owner action, no branch</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>Owner decision D2</t>
+        </is>
+      </c>
+      <c r="M93" t="inlineStr">
+        <is>
+          <t>Default branch main; development exists</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="17" t="inlineStr">
+        <is>
+          <t>LS-039</t>
+        </is>
+      </c>
+      <c r="B94" s="61" t="inlineStr">
+        <is>
+          <t>Build verification environment (ADR-017)</t>
+        </is>
+      </c>
+      <c r="C94" s="4" t="inlineStr">
+        <is>
+          <t>LS-009</t>
+        </is>
+      </c>
+      <c r="D94" s="62" t="inlineStr">
+        <is>
+          <t>LS-009</t>
+        </is>
+      </c>
+      <c r="E94" s="62" t="inlineStr">
+        <is>
+          <t>LS-030, LS-035, LS-130</t>
+        </is>
+      </c>
+      <c r="F94" s="62" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G94" s="62" t="inlineStr">
+        <is>
+          <t>Cloud environment settings</t>
+        </is>
+      </c>
+      <c r="H94" s="61" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>P2 entry</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>Owner action, no branch</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>Owner decision D3</t>
+        </is>
+      </c>
+      <c r="M94" t="inlineStr">
+        <is>
+          <t>Gradle sync downloading AGP succeeds</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M83"/>
+  <autoFilter ref="A1:M94"/>
   <mergeCells count="14">
     <mergeCell ref="A92:B92"/>
     <mergeCell ref="A86:B86"/>
@@ -14641,7 +15383,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -14737,7 +15479,7 @@
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Pending toolchain check (LS-001)</t>
+          <t>Recommended: Navigation Compose type-safe routes; re-check Navigation 3 in LS-030</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
@@ -14790,7 +15532,7 @@
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>app, core:designsystem, core:ui, core:common, domain, data, feature:{onboarding,home,discover,storydetails,create,reader,player,library,settings,profiles,notifications,subscription}</t>
+          <t>Recommended (D4): 7 feature modules — onboarding, home, discover, create, reader, library, settings — plus app, build-logic, core:designsystem, core:ui, core:common, domain, data</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
@@ -15267,7 +16009,7 @@
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Decide after LS-001 toolchain check</t>
+          <t>Recommended (D7): Roborazzi; Compose Preview Screenshot Testing as alternative</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
@@ -15479,7 +16221,7 @@
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>Pending owner decision (LS-004)</t>
+          <t>Recommended (D13): settings UI only in MVP; real local notification is a separate approved ticket</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
@@ -15509,8 +16251,179 @@
         </is>
       </c>
     </row>
+    <row r="17" ht="31" customHeight="1">
+      <c r="A17" s="17" t="inlineStr">
+        <is>
+          <t>ADR-016</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Minimum SDK</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Compatibility for Kannada rendering and per-app language</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>minSdk 24 · 26 · 28</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>Recommended (D5): minSdk 26</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>Predictable font + per-app-language behaviour; AppCompat backport below Android 13</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>Android 7.x unsupported</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="I17" s="4" t="inlineStr">
+        <is>
+          <t>Project owner</t>
+        </is>
+      </c>
+      <c r="J17" s="4" t="inlineStr">
+        <is>
+          <t>29 Oct 2026</t>
+        </is>
+      </c>
+      <c r="K17" s="4" t="inlineStr">
+        <is>
+          <t>LS-030, LS-040</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="31" customHeight="1">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>ADR-017</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Build and test verification environment</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Cloud agent workspace cannot reach dl.google.com (R-21)</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Allow host · CI only · owner machine only</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Recommended (D3): allow dl.google.com + GitHub Actions on every PR</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>PRs need real build evidence</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>CI becomes part of the foundation milestone</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="I18" s="4" t="inlineStr">
+        <is>
+          <t>Project owner</t>
+        </is>
+      </c>
+      <c r="J18" s="4" t="inlineStr">
+        <is>
+          <t>29 Oct 2026</t>
+        </is>
+      </c>
+      <c r="K18" s="4" t="inlineStr">
+        <is>
+          <t>LS-039, LS-130</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="31" customHeight="1">
+      <c r="A19" s="17" t="inlineStr">
+        <is>
+          <t>ADR-018</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Static analysis</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>No-hardcoding policy needs enforcement</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>Lint only · Lint + Detekt · Lint + Detekt + ktlint</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>Recommended (D15): Lint (errors) + Detekt + ktlint</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>Catches magic numbers, raw colours/dp and style drift</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>Rules maintained in build-logic</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="I19" s="4" t="inlineStr">
+        <is>
+          <t>Project owner</t>
+        </is>
+      </c>
+      <c r="J19" s="4" t="inlineStr">
+        <is>
+          <t>29 Oct 2026</t>
+        </is>
+      </c>
+      <c r="K19" s="4" t="inlineStr">
+        <is>
+          <t>LS-034</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K16"/>
+  <autoFilter ref="A1:K19"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -15522,7 +16435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K21"/>
+  <dimension ref="A1:K25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -15955,7 +16868,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>#716B80 on cream at 10–12px and #817B8D nav labels likely &lt; 4.5:1</t>
+          <t>Measured 29 Oct 2026 (docs/design/accessibility-spec.md): muted #716B80 passes (4.87:1 on cream, 5.10:1 on white); nav-inactive #817B8D fails (3.89:1 on cream), lavender focus ring on white 2.53:1 and progress fill on track 2.02:1 fail non-text 3:1</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
@@ -15970,7 +16883,7 @@
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>Measure; adjust token or size</t>
+          <t>Darken nav-inactive token; thicker/darker focus ring and progress fill</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
@@ -16540,7 +17453,7 @@
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>Run P0 first; no assumptions</t>
+          <t>Closed by P0 assessment 29 Oct 2026: repo is docs-only (see R-21, R-22)</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
@@ -16560,7 +17473,7 @@
       </c>
       <c r="K18" s="4" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -16735,8 +17648,236 @@
         </is>
       </c>
     </row>
+    <row r="22" ht="18" customHeight="1">
+      <c r="A22" s="17" t="inlineStr">
+        <is>
+          <t>R-21</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Build environment blocked</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Delivery</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>Cloud agent workspace gets 403 for dl.google.com (Google Maven, Android SDK); agents cannot build Android there</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>Allow dl.google.com in cloud environment; GitHub Actions CI; no unverified build claims (ADR-017, LS-039)</t>
+        </is>
+      </c>
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="I22" s="4" t="inlineStr">
+        <is>
+          <t>Choose build environment (D3)</t>
+        </is>
+      </c>
+      <c r="J22" s="4" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="K22" s="4" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="18" customHeight="1">
+      <c r="A23" s="17" t="inlineStr">
+        <is>
+          <t>R-22</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Default branch misconfigured</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Delivery</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>GitHub default branch is the docs branch claude/project-thread-sszyf7, not main</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>Owner merges PR #1, sets default to main, creates development (LS-009)</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="I23" s="4" t="inlineStr">
+        <is>
+          <t>Approve repo hygiene (D2)</t>
+        </is>
+      </c>
+      <c r="J23" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K23" s="4" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="18" customHeight="1">
+      <c r="A24" s="17" t="inlineStr">
+        <is>
+          <t>R-23</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Design drift</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>Agents cannot re-read the Figma Make file; docs/design/ is a 29 Oct 2026 snapshot</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>Owner flags Make changes; re-export the design pack</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="I24" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J24" s="4" t="inlineStr">
+        <is>
+          <t>P1–P7</t>
+        </is>
+      </c>
+      <c r="K24" s="4" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="17" t="inlineStr">
+        <is>
+          <t>R-24</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>Public repository</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>Repository is public; secrets or child data committed would be exposed</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>Secret scanning in CI; .gitignore local.properties/keystores; synthetic data only</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>Security Reviewer</t>
+        </is>
+      </c>
+      <c r="I25" s="4" t="inlineStr">
+        <is>
+          <t>Keep public or make private</t>
+        </is>
+      </c>
+      <c r="J25" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K25" s="4" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K21"/>
+  <autoFilter ref="A1:K25"/>
   <conditionalFormatting sqref="E2:E21">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="3">
       <formula>"High"</formula>
@@ -16758,7 +17899,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P83"/>
+  <dimension ref="A1:P85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -23177,6 +24318,170 @@
       <c r="P83" s="4" t="inlineStr">
         <is>
           <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="17" t="inlineStr">
+        <is>
+          <t>LS-009</t>
+        </is>
+      </c>
+      <c r="B84" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C84" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D84" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E84" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F84" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G84" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H84" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I84" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J84" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K84" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L84" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M84" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N84" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O84" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P84" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="17" t="inlineStr">
+        <is>
+          <t>LS-039</t>
+        </is>
+      </c>
+      <c r="B85" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C85" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D85" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E85" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F85" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G85" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H85" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I85" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J85" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K85" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L85" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M85" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N85" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O85" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P85" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -23278,7 +24583,7 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>core:common · strings.xml</t>
+          <t>app · strings.xml</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
@@ -23313,7 +24618,7 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>core:common · strings.xml</t>
+          <t>core:ui · strings.xml</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
@@ -25063,7 +26368,7 @@
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>core:common · strings.xml</t>
+          <t>core:ui · strings.xml</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr">
@@ -25098,7 +26403,7 @@
       </c>
       <c r="B54" s="4" t="inlineStr">
         <is>
-          <t>core:common · strings.xml</t>
+          <t>core:ui · strings.xml</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr">
@@ -25133,7 +26438,7 @@
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>core:common · strings.xml</t>
+          <t>core:ui · strings.xml</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
@@ -25168,7 +26473,7 @@
       </c>
       <c r="B56" s="4" t="inlineStr">
         <is>
-          <t>core:common · strings.xml</t>
+          <t>core:ui · strings.xml</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr">
@@ -25203,7 +26508,7 @@
       </c>
       <c r="B57" s="4" t="inlineStr">
         <is>
-          <t>core:common · strings.xml</t>
+          <t>core:ui · strings.xml</t>
         </is>
       </c>
       <c r="C57" s="4" t="inlineStr">
@@ -25238,7 +26543,7 @@
       </c>
       <c r="B58" s="4" t="inlineStr">
         <is>
-          <t>core:common · strings.xml</t>
+          <t>core:ui · strings.xml</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
@@ -25798,7 +27103,7 @@
       </c>
       <c r="B74" s="4" t="inlineStr">
         <is>
-          <t>core:common · strings.xml</t>
+          <t>core:ui · strings.xml</t>
         </is>
       </c>
       <c r="C74" s="4" t="inlineStr">
@@ -25833,7 +27138,7 @@
       </c>
       <c r="B75" s="4" t="inlineStr">
         <is>
-          <t>core:common · strings.xml</t>
+          <t>core:ui · strings.xml</t>
         </is>
       </c>
       <c r="C75" s="4" t="inlineStr">
@@ -25868,7 +27173,7 @@
       </c>
       <c r="B76" s="4" t="inlineStr">
         <is>
-          <t>core:common · strings.xml</t>
+          <t>core:ui · strings.xml</t>
         </is>
       </c>
       <c r="C76" s="4" t="inlineStr">
@@ -25903,7 +27208,7 @@
       </c>
       <c r="B77" s="4" t="inlineStr">
         <is>
-          <t>core:common · strings.xml</t>
+          <t>core:ui · strings.xml</t>
         </is>
       </c>
       <c r="C77" s="4" t="inlineStr">
@@ -25938,7 +27243,7 @@
       </c>
       <c r="B78" s="4" t="inlineStr">
         <is>
-          <t>core:common · strings.xml</t>
+          <t>core:ui · strings.xml</t>
         </is>
       </c>
       <c r="C78" s="4" t="inlineStr">
@@ -25973,7 +27278,7 @@
       </c>
       <c r="B79" s="4" t="inlineStr">
         <is>
-          <t>core:common · strings.xml</t>
+          <t>core:ui · strings.xml</t>
         </is>
       </c>
       <c r="C79" s="4" t="inlineStr">
@@ -26008,7 +27313,7 @@
       </c>
       <c r="B80" s="4" t="inlineStr">
         <is>
-          <t>core:common · strings.xml</t>
+          <t>core:ui · strings.xml</t>
         </is>
       </c>
       <c r="C80" s="4" t="inlineStr">
@@ -26043,7 +27348,7 @@
       </c>
       <c r="B81" s="4" t="inlineStr">
         <is>
-          <t>core:common · strings.xml</t>
+          <t>core:ui · strings.xml</t>
         </is>
       </c>
       <c r="C81" s="4" t="inlineStr">
@@ -26078,7 +27383,7 @@
       </c>
       <c r="B82" s="4" t="inlineStr">
         <is>
-          <t>core:common · strings.xml</t>
+          <t>core:ui · strings.xml</t>
         </is>
       </c>
       <c r="C82" s="4" t="inlineStr">
@@ -26113,7 +27418,7 @@
       </c>
       <c r="B83" s="4" t="inlineStr">
         <is>
-          <t>core:common · strings.xml</t>
+          <t>core:ui · strings.xml</t>
         </is>
       </c>
       <c r="C83" s="4" t="inlineStr">
@@ -26148,7 +27453,7 @@
       </c>
       <c r="B84" s="4" t="inlineStr">
         <is>
-          <t>core:common · strings.xml</t>
+          <t>core:ui · strings.xml</t>
         </is>
       </c>
       <c r="C84" s="4" t="inlineStr">
@@ -26183,7 +27488,7 @@
       </c>
       <c r="B85" s="4" t="inlineStr">
         <is>
-          <t>core:common · strings.xml</t>
+          <t>core:ui · strings.xml</t>
         </is>
       </c>
       <c r="C85" s="4" t="inlineStr">
@@ -26778,7 +28083,7 @@
       </c>
       <c r="B102" s="4" t="inlineStr">
         <is>
-          <t>feature:storydetails · strings.xml</t>
+          <t>feature:discover · strings.xml</t>
         </is>
       </c>
       <c r="C102" s="4" t="inlineStr">
@@ -26813,7 +28118,7 @@
       </c>
       <c r="B103" s="4" t="inlineStr">
         <is>
-          <t>feature:storydetails · strings.xml</t>
+          <t>feature:discover · strings.xml</t>
         </is>
       </c>
       <c r="C103" s="4" t="inlineStr">
@@ -26848,7 +28153,7 @@
       </c>
       <c r="B104" s="4" t="inlineStr">
         <is>
-          <t>feature:storydetails · strings.xml</t>
+          <t>feature:discover · strings.xml</t>
         </is>
       </c>
       <c r="C104" s="4" t="inlineStr">
@@ -26883,7 +28188,7 @@
       </c>
       <c r="B105" s="4" t="inlineStr">
         <is>
-          <t>feature:storydetails · strings.xml</t>
+          <t>feature:discover · strings.xml</t>
         </is>
       </c>
       <c r="C105" s="4" t="inlineStr">
@@ -26918,7 +28223,7 @@
       </c>
       <c r="B106" s="4" t="inlineStr">
         <is>
-          <t>feature:storydetails · strings.xml</t>
+          <t>feature:discover · strings.xml</t>
         </is>
       </c>
       <c r="C106" s="4" t="inlineStr">
@@ -28878,7 +30183,7 @@
       </c>
       <c r="B162" s="4" t="inlineStr">
         <is>
-          <t>feature:player · strings.xml</t>
+          <t>feature:reader · strings.xml</t>
         </is>
       </c>
       <c r="C162" s="4" t="inlineStr">
@@ -28913,7 +30218,7 @@
       </c>
       <c r="B163" s="4" t="inlineStr">
         <is>
-          <t>feature:player · strings.xml</t>
+          <t>feature:reader · strings.xml</t>
         </is>
       </c>
       <c r="C163" s="4" t="inlineStr">
@@ -28948,7 +30253,7 @@
       </c>
       <c r="B164" s="4" t="inlineStr">
         <is>
-          <t>feature:player · strings.xml</t>
+          <t>feature:reader · strings.xml</t>
         </is>
       </c>
       <c r="C164" s="4" t="inlineStr">
@@ -28983,7 +30288,7 @@
       </c>
       <c r="B165" s="4" t="inlineStr">
         <is>
-          <t>feature:player · strings.xml</t>
+          <t>feature:reader · strings.xml</t>
         </is>
       </c>
       <c r="C165" s="4" t="inlineStr">
@@ -29018,7 +30323,7 @@
       </c>
       <c r="B166" s="4" t="inlineStr">
         <is>
-          <t>feature:player · strings.xml</t>
+          <t>feature:reader · strings.xml</t>
         </is>
       </c>
       <c r="C166" s="4" t="inlineStr">
@@ -29053,7 +30358,7 @@
       </c>
       <c r="B167" s="4" t="inlineStr">
         <is>
-          <t>feature:player · strings.xml</t>
+          <t>feature:reader · strings.xml</t>
         </is>
       </c>
       <c r="C167" s="4" t="inlineStr">
@@ -29088,7 +30393,7 @@
       </c>
       <c r="B168" s="4" t="inlineStr">
         <is>
-          <t>feature:player · strings.xml</t>
+          <t>feature:reader · strings.xml</t>
         </is>
       </c>
       <c r="C168" s="4" t="inlineStr">
@@ -29123,7 +30428,7 @@
       </c>
       <c r="B169" s="4" t="inlineStr">
         <is>
-          <t>feature:player · strings.xml</t>
+          <t>feature:reader · strings.xml</t>
         </is>
       </c>
       <c r="C169" s="4" t="inlineStr">
@@ -29158,7 +30463,7 @@
       </c>
       <c r="B170" s="4" t="inlineStr">
         <is>
-          <t>feature:player · strings.xml</t>
+          <t>feature:reader · strings.xml</t>
         </is>
       </c>
       <c r="C170" s="4" t="inlineStr">
@@ -29193,7 +30498,7 @@
       </c>
       <c r="B171" s="4" t="inlineStr">
         <is>
-          <t>feature:player · strings.xml</t>
+          <t>feature:reader · strings.xml</t>
         </is>
       </c>
       <c r="C171" s="4" t="inlineStr">
@@ -29228,7 +30533,7 @@
       </c>
       <c r="B172" s="4" t="inlineStr">
         <is>
-          <t>feature:player · strings.xml</t>
+          <t>feature:reader · strings.xml</t>
         </is>
       </c>
       <c r="C172" s="4" t="inlineStr">
@@ -29263,7 +30568,7 @@
       </c>
       <c r="B173" s="4" t="inlineStr">
         <is>
-          <t>feature:player · strings.xml</t>
+          <t>feature:reader · strings.xml</t>
         </is>
       </c>
       <c r="C173" s="4" t="inlineStr">
@@ -29298,7 +30603,7 @@
       </c>
       <c r="B174" s="4" t="inlineStr">
         <is>
-          <t>feature:player · strings.xml</t>
+          <t>feature:reader · strings.xml</t>
         </is>
       </c>
       <c r="C174" s="4" t="inlineStr">
@@ -29333,7 +30638,7 @@
       </c>
       <c r="B175" s="4" t="inlineStr">
         <is>
-          <t>feature:player · strings.xml</t>
+          <t>feature:reader · strings.xml</t>
         </is>
       </c>
       <c r="C175" s="4" t="inlineStr">
@@ -29368,7 +30673,7 @@
       </c>
       <c r="B176" s="4" t="inlineStr">
         <is>
-          <t>feature:player · strings.xml</t>
+          <t>feature:reader · strings.xml</t>
         </is>
       </c>
       <c r="C176" s="4" t="inlineStr">
@@ -29403,7 +30708,7 @@
       </c>
       <c r="B177" s="4" t="inlineStr">
         <is>
-          <t>feature:player · strings.xml</t>
+          <t>feature:reader · strings.xml</t>
         </is>
       </c>
       <c r="C177" s="4" t="inlineStr">
@@ -29438,7 +30743,7 @@
       </c>
       <c r="B178" s="4" t="inlineStr">
         <is>
-          <t>feature:player · strings.xml</t>
+          <t>feature:reader · strings.xml</t>
         </is>
       </c>
       <c r="C178" s="4" t="inlineStr">
@@ -30908,7 +32213,7 @@
       </c>
       <c r="B220" s="4" t="inlineStr">
         <is>
-          <t>feature:profiles · strings.xml</t>
+          <t>feature:settings · strings.xml</t>
         </is>
       </c>
       <c r="C220" s="4" t="inlineStr">
@@ -30943,7 +32248,7 @@
       </c>
       <c r="B221" s="4" t="inlineStr">
         <is>
-          <t>feature:profiles · strings.xml</t>
+          <t>feature:settings · strings.xml</t>
         </is>
       </c>
       <c r="C221" s="4" t="inlineStr">
@@ -30978,7 +32283,7 @@
       </c>
       <c r="B222" s="4" t="inlineStr">
         <is>
-          <t>feature:profiles · strings.xml</t>
+          <t>feature:settings · strings.xml</t>
         </is>
       </c>
       <c r="C222" s="4" t="inlineStr">
@@ -31013,7 +32318,7 @@
       </c>
       <c r="B223" s="4" t="inlineStr">
         <is>
-          <t>feature:profiles · strings.xml</t>
+          <t>feature:settings · strings.xml</t>
         </is>
       </c>
       <c r="C223" s="4" t="inlineStr">
@@ -31048,7 +32353,7 @@
       </c>
       <c r="B224" s="4" t="inlineStr">
         <is>
-          <t>feature:profiles · strings.xml</t>
+          <t>feature:settings · strings.xml</t>
         </is>
       </c>
       <c r="C224" s="4" t="inlineStr">
@@ -31083,7 +32388,7 @@
       </c>
       <c r="B225" s="4" t="inlineStr">
         <is>
-          <t>feature:profiles · strings.xml</t>
+          <t>feature:settings · strings.xml</t>
         </is>
       </c>
       <c r="C225" s="4" t="inlineStr">
@@ -31118,7 +32423,7 @@
       </c>
       <c r="B226" s="4" t="inlineStr">
         <is>
-          <t>feature:profiles · strings.xml</t>
+          <t>feature:settings · strings.xml</t>
         </is>
       </c>
       <c r="C226" s="4" t="inlineStr">
@@ -31153,7 +32458,7 @@
       </c>
       <c r="B227" s="4" t="inlineStr">
         <is>
-          <t>feature:profiles · strings.xml</t>
+          <t>feature:settings · strings.xml</t>
         </is>
       </c>
       <c r="C227" s="4" t="inlineStr">
@@ -31188,7 +32493,7 @@
       </c>
       <c r="B228" s="4" t="inlineStr">
         <is>
-          <t>feature:profiles · strings.xml</t>
+          <t>feature:settings · strings.xml</t>
         </is>
       </c>
       <c r="C228" s="4" t="inlineStr">
@@ -31223,7 +32528,7 @@
       </c>
       <c r="B229" s="4" t="inlineStr">
         <is>
-          <t>feature:profiles · strings.xml</t>
+          <t>feature:settings · strings.xml</t>
         </is>
       </c>
       <c r="C229" s="4" t="inlineStr">
@@ -31258,7 +32563,7 @@
       </c>
       <c r="B230" s="4" t="inlineStr">
         <is>
-          <t>feature:subscription · strings.xml</t>
+          <t>feature:settings · strings.xml</t>
         </is>
       </c>
       <c r="C230" s="4" t="inlineStr">
@@ -31293,7 +32598,7 @@
       </c>
       <c r="B231" s="4" t="inlineStr">
         <is>
-          <t>feature:subscription · strings.xml</t>
+          <t>feature:settings · strings.xml</t>
         </is>
       </c>
       <c r="C231" s="4" t="inlineStr">
@@ -31328,7 +32633,7 @@
       </c>
       <c r="B232" s="4" t="inlineStr">
         <is>
-          <t>feature:subscription · strings.xml</t>
+          <t>feature:settings · strings.xml</t>
         </is>
       </c>
       <c r="C232" s="4" t="inlineStr">
@@ -31363,7 +32668,7 @@
       </c>
       <c r="B233" s="4" t="inlineStr">
         <is>
-          <t>feature:subscription · strings.xml</t>
+          <t>feature:settings · strings.xml</t>
         </is>
       </c>
       <c r="C233" s="4" t="inlineStr">
@@ -31398,7 +32703,7 @@
       </c>
       <c r="B234" s="4" t="inlineStr">
         <is>
-          <t>feature:subscription · strings.xml</t>
+          <t>feature:settings · strings.xml</t>
         </is>
       </c>
       <c r="C234" s="4" t="inlineStr">
@@ -31433,7 +32738,7 @@
       </c>
       <c r="B235" s="4" t="inlineStr">
         <is>
-          <t>feature:subscription · strings.xml</t>
+          <t>feature:settings · strings.xml</t>
         </is>
       </c>
       <c r="C235" s="4" t="inlineStr">
@@ -31468,7 +32773,7 @@
       </c>
       <c r="B236" s="4" t="inlineStr">
         <is>
-          <t>feature:subscription · strings.xml</t>
+          <t>feature:settings · strings.xml</t>
         </is>
       </c>
       <c r="C236" s="4" t="inlineStr">
@@ -31503,7 +32808,7 @@
       </c>
       <c r="B237" s="4" t="inlineStr">
         <is>
-          <t>feature:subscription · strings.xml</t>
+          <t>feature:settings · strings.xml</t>
         </is>
       </c>
       <c r="C237" s="4" t="inlineStr">
@@ -31538,7 +32843,7 @@
       </c>
       <c r="B238" s="4" t="inlineStr">
         <is>
-          <t>feature:subscription · strings.xml</t>
+          <t>feature:settings · strings.xml</t>
         </is>
       </c>
       <c r="C238" s="4" t="inlineStr">
@@ -31573,7 +32878,7 @@
       </c>
       <c r="B239" s="4" t="inlineStr">
         <is>
-          <t>feature:subscription · strings.xml</t>
+          <t>feature:settings · strings.xml</t>
         </is>
       </c>
       <c r="C239" s="4" t="inlineStr">
@@ -31608,7 +32913,7 @@
       </c>
       <c r="B240" s="4" t="inlineStr">
         <is>
-          <t>feature:subscription · strings.xml</t>
+          <t>feature:settings · strings.xml</t>
         </is>
       </c>
       <c r="C240" s="4" t="inlineStr">
@@ -31643,7 +32948,7 @@
       </c>
       <c r="B241" s="4" t="inlineStr">
         <is>
-          <t>feature:subscription · strings.xml</t>
+          <t>feature:settings · strings.xml</t>
         </is>
       </c>
       <c r="C241" s="4" t="inlineStr">
@@ -31678,7 +32983,7 @@
       </c>
       <c r="B242" s="4" t="inlineStr">
         <is>
-          <t>feature:subscription · strings.xml</t>
+          <t>feature:settings · strings.xml</t>
         </is>
       </c>
       <c r="C242" s="4" t="inlineStr">
@@ -31713,7 +33018,7 @@
       </c>
       <c r="B243" s="4" t="inlineStr">
         <is>
-          <t>feature:subscription · strings.xml</t>
+          <t>feature:settings · strings.xml</t>
         </is>
       </c>
       <c r="C243" s="4" t="inlineStr">
@@ -31748,7 +33053,7 @@
       </c>
       <c r="B244" s="4" t="inlineStr">
         <is>
-          <t>feature:subscription · strings.xml</t>
+          <t>feature:settings · strings.xml</t>
         </is>
       </c>
       <c r="C244" s="4" t="inlineStr">
@@ -31783,7 +33088,7 @@
       </c>
       <c r="B245" s="4" t="inlineStr">
         <is>
-          <t>feature:subscription · strings.xml</t>
+          <t>feature:settings · strings.xml</t>
         </is>
       </c>
       <c r="C245" s="4" t="inlineStr">
@@ -31818,7 +33123,7 @@
       </c>
       <c r="B246" s="4" t="inlineStr">
         <is>
-          <t>feature:subscription · strings.xml</t>
+          <t>feature:settings · strings.xml</t>
         </is>
       </c>
       <c r="C246" s="4" t="inlineStr">
@@ -31853,7 +33158,7 @@
       </c>
       <c r="B247" s="4" t="inlineStr">
         <is>
-          <t>feature:subscription · strings.xml</t>
+          <t>feature:settings · strings.xml</t>
         </is>
       </c>
       <c r="C247" s="4" t="inlineStr">
@@ -31888,7 +33193,7 @@
       </c>
       <c r="B248" s="4" t="inlineStr">
         <is>
-          <t>feature:subscription · strings.xml</t>
+          <t>feature:settings · strings.xml</t>
         </is>
       </c>
       <c r="C248" s="4" t="inlineStr">
@@ -31923,7 +33228,7 @@
       </c>
       <c r="B249" s="4" t="inlineStr">
         <is>
-          <t>feature:subscription · strings.xml</t>
+          <t>feature:settings · strings.xml</t>
         </is>
       </c>
       <c r="C249" s="4" t="inlineStr">
@@ -31958,7 +33263,7 @@
       </c>
       <c r="B250" s="4" t="inlineStr">
         <is>
-          <t>feature:subscription · strings.xml</t>
+          <t>feature:settings · strings.xml</t>
         </is>
       </c>
       <c r="C250" s="4" t="inlineStr">
@@ -31993,7 +33298,7 @@
       </c>
       <c r="B251" s="4" t="inlineStr">
         <is>
-          <t>feature:subscription · strings.xml</t>
+          <t>feature:settings · strings.xml</t>
         </is>
       </c>
       <c r="C251" s="4" t="inlineStr">
@@ -32028,7 +33333,7 @@
       </c>
       <c r="B252" s="4" t="inlineStr">
         <is>
-          <t>feature:subscription · strings.xml</t>
+          <t>feature:settings · strings.xml</t>
         </is>
       </c>
       <c r="C252" s="4" t="inlineStr">
@@ -32063,7 +33368,7 @@
       </c>
       <c r="B253" s="4" t="inlineStr">
         <is>
-          <t>feature:subscription · strings.xml</t>
+          <t>feature:settings · strings.xml</t>
         </is>
       </c>
       <c r="C253" s="4" t="inlineStr">
@@ -32098,7 +33403,7 @@
       </c>
       <c r="B254" s="4" t="inlineStr">
         <is>
-          <t>feature:subscription · strings.xml</t>
+          <t>feature:settings · strings.xml</t>
         </is>
       </c>
       <c r="C254" s="4" t="inlineStr">
@@ -32133,7 +33438,7 @@
       </c>
       <c r="B255" s="4" t="inlineStr">
         <is>
-          <t>feature:subscription · strings.xml</t>
+          <t>feature:settings · strings.xml</t>
         </is>
       </c>
       <c r="C255" s="4" t="inlineStr">
@@ -32938,7 +34243,7 @@
       </c>
       <c r="B278" s="4" t="inlineStr">
         <is>
-          <t>feature:notifications · strings.xml</t>
+          <t>feature:settings · strings.xml</t>
         </is>
       </c>
       <c r="C278" s="4" t="inlineStr">
@@ -32973,7 +34278,7 @@
       </c>
       <c r="B279" s="4" t="inlineStr">
         <is>
-          <t>feature:notifications · strings.xml</t>
+          <t>feature:settings · strings.xml</t>
         </is>
       </c>
       <c r="C279" s="4" t="inlineStr">
@@ -33008,7 +34313,7 @@
       </c>
       <c r="B280" s="4" t="inlineStr">
         <is>
-          <t>feature:notifications · strings.xml</t>
+          <t>feature:settings · strings.xml</t>
         </is>
       </c>
       <c r="C280" s="4" t="inlineStr">
@@ -33043,7 +34348,7 @@
       </c>
       <c r="B281" s="4" t="inlineStr">
         <is>
-          <t>feature:notifications · strings.xml</t>
+          <t>feature:settings · strings.xml</t>
         </is>
       </c>
       <c r="C281" s="4" t="inlineStr">
@@ -33078,7 +34383,7 @@
       </c>
       <c r="B282" s="4" t="inlineStr">
         <is>
-          <t>feature:notifications · strings.xml</t>
+          <t>feature:settings · strings.xml</t>
         </is>
       </c>
       <c r="C282" s="4" t="inlineStr">
@@ -37797,7 +39102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL83"/>
+  <dimension ref="A1:AL85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -38132,7 +39437,11 @@
           <t>N/A (read-only) – verify `git status` unchanged</t>
         </is>
       </c>
-      <c r="T2" s="4" t="inlineStr"/>
+      <c r="T2" s="4" t="inlineStr">
+        <is>
+          <t>Read-only: git/GitHub inspection, Figma whoami, network probes</t>
+        </is>
+      </c>
       <c r="U2" s="4" t="n">
         <v>3</v>
       </c>
@@ -38170,7 +39479,7 @@
       <c r="AC2" s="4" t="inlineStr"/>
       <c r="AD2" s="4" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="AE2" s="4" t="inlineStr">
@@ -38180,10 +39489,14 @@
       </c>
       <c r="AF2" s="4" t="inlineStr">
         <is>
-          <t>Approval A (read-only)</t>
-        </is>
-      </c>
-      <c r="AG2" s="4" t="inlineStr"/>
+          <t>Approval A — report delivered</t>
+        </is>
+      </c>
+      <c r="AG2" s="4" t="inlineStr">
+        <is>
+          <t>P0 assessment delivered 29 Oct 2026 (Claude Doc "LittleStory — P0 Discovery Assessment"): repo docs-only, default branch misconfigured, Figma Make not readable by agents, cloud workspace cannot reach dl.google.com.</t>
+        </is>
+      </c>
       <c r="AH2" s="4" t="inlineStr">
         <is>
           <t>None</t>
@@ -38525,14 +39838,14 @@
       </c>
       <c r="AA4" s="4" t="inlineStr">
         <is>
-          <t>feature/LS-003-requirements-catalogue-user-journeys-a</t>
+          <t>claude/project-thread-veobz7</t>
         </is>
       </c>
       <c r="AB4" s="4" t="inlineStr"/>
       <c r="AC4" s="4" t="inlineStr"/>
       <c r="AD4" s="4" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>In Review</t>
         </is>
       </c>
       <c r="AE4" s="4" t="inlineStr">
@@ -38542,10 +39855,14 @@
       </c>
       <c r="AF4" s="4" t="inlineStr">
         <is>
-          <t>Awaiting Approval B</t>
-        </is>
-      </c>
-      <c r="AG4" s="4" t="inlineStr"/>
+          <t>Approval B granted — awaiting owner review of docs PR</t>
+        </is>
+      </c>
+      <c r="AG4" s="4" t="inlineStr">
+        <is>
+          <t>Drafted 29 Oct 2026: docs/product/*</t>
+        </is>
+      </c>
       <c r="AH4" s="4" t="inlineStr">
         <is>
           <t>None</t>
@@ -38697,14 +40014,14 @@
       </c>
       <c r="AA5" s="4" t="inlineStr">
         <is>
-          <t>feature/LS-004-resolve-design-gaps-open-product</t>
+          <t>claude/project-thread-veobz7</t>
         </is>
       </c>
       <c r="AB5" s="4" t="inlineStr"/>
       <c r="AC5" s="4" t="inlineStr"/>
       <c r="AD5" s="4" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>In Review</t>
         </is>
       </c>
       <c r="AE5" s="4" t="inlineStr">
@@ -38714,10 +40031,14 @@
       </c>
       <c r="AF5" s="4" t="inlineStr">
         <is>
-          <t>Awaiting Approval B</t>
-        </is>
-      </c>
-      <c r="AG5" s="4" t="inlineStr"/>
+          <t>Approval B granted — awaiting owner review of docs PR</t>
+        </is>
+      </c>
+      <c r="AG5" s="4" t="inlineStr">
+        <is>
+          <t>Drafted 29 Oct 2026: docs/project-management/decision-log.md (D10, D13), docs/design/figma-audit.md</t>
+        </is>
+      </c>
       <c r="AH5" s="4" t="inlineStr">
         <is>
           <t>None</t>
@@ -38873,14 +40194,14 @@
       </c>
       <c r="AA6" s="4" t="inlineStr">
         <is>
-          <t>feature/LS-005-claude-md-and-github-copilot</t>
+          <t>claude/project-thread-veobz7</t>
         </is>
       </c>
       <c r="AB6" s="4" t="inlineStr"/>
       <c r="AC6" s="4" t="inlineStr"/>
       <c r="AD6" s="4" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>In Review</t>
         </is>
       </c>
       <c r="AE6" s="4" t="inlineStr">
@@ -38890,10 +40211,14 @@
       </c>
       <c r="AF6" s="4" t="inlineStr">
         <is>
-          <t>Awaiting Approval B</t>
-        </is>
-      </c>
-      <c r="AG6" s="4" t="inlineStr"/>
+          <t>Approval B granted — awaiting owner review of docs PR</t>
+        </is>
+      </c>
+      <c r="AG6" s="4" t="inlineStr">
+        <is>
+          <t>Drafted 29 Oct 2026: CLAUDE.md, .github/copilot-instructions.md</t>
+        </is>
+      </c>
       <c r="AH6" s="4" t="inlineStr">
         <is>
           <t>None</t>
@@ -39044,14 +40369,14 @@
       </c>
       <c r="AA7" s="4" t="inlineStr">
         <is>
-          <t>feature/LS-006-prompt-library-prompts-00-21</t>
+          <t>claude/project-thread-veobz7</t>
         </is>
       </c>
       <c r="AB7" s="4" t="inlineStr"/>
       <c r="AC7" s="4" t="inlineStr"/>
       <c r="AD7" s="4" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>In Review</t>
         </is>
       </c>
       <c r="AE7" s="4" t="inlineStr">
@@ -39061,10 +40386,14 @@
       </c>
       <c r="AF7" s="4" t="inlineStr">
         <is>
-          <t>Awaiting Approval B</t>
-        </is>
-      </c>
-      <c r="AG7" s="4" t="inlineStr"/>
+          <t>Approval B granted — awaiting owner review of docs PR</t>
+        </is>
+      </c>
+      <c r="AG7" s="4" t="inlineStr">
+        <is>
+          <t>Drafted 29 Oct 2026: prompts/00–21, prompts/tickets/ (P2)</t>
+        </is>
+      </c>
       <c r="AH7" s="4" t="inlineStr">
         <is>
           <t>None</t>
@@ -39212,14 +40541,14 @@
       </c>
       <c r="AA8" s="4" t="inlineStr">
         <is>
-          <t>feature/LS-007-commit-backlog-workbook-and-design</t>
+          <t>claude/project-thread-veobz7</t>
         </is>
       </c>
       <c r="AB8" s="4" t="inlineStr"/>
       <c r="AC8" s="4" t="inlineStr"/>
       <c r="AD8" s="4" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>In Review</t>
         </is>
       </c>
       <c r="AE8" s="4" t="inlineStr">
@@ -39229,10 +40558,14 @@
       </c>
       <c r="AF8" s="4" t="inlineStr">
         <is>
-          <t>Awaiting Approval B</t>
-        </is>
-      </c>
-      <c r="AG8" s="4" t="inlineStr"/>
+          <t>Approval B granted — awaiting owner review of docs PR</t>
+        </is>
+      </c>
+      <c r="AG8" s="4" t="inlineStr">
+        <is>
+          <t>Drafted 29 Oct 2026: docs/ (design pack in PR #1)</t>
+        </is>
+      </c>
       <c r="AH8" s="4" t="inlineStr">
         <is>
           <t>None</t>
@@ -39380,14 +40713,14 @@
       </c>
       <c r="AA9" s="4" t="inlineStr">
         <is>
-          <t>feature/LS-008-architecture-adrs-adr-001-015</t>
+          <t>claude/project-thread-veobz7</t>
         </is>
       </c>
       <c r="AB9" s="4" t="inlineStr"/>
       <c r="AC9" s="4" t="inlineStr"/>
       <c r="AD9" s="4" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>In Review</t>
         </is>
       </c>
       <c r="AE9" s="4" t="inlineStr">
@@ -39397,10 +40730,14 @@
       </c>
       <c r="AF9" s="4" t="inlineStr">
         <is>
-          <t>Awaiting Approval B</t>
-        </is>
-      </c>
-      <c r="AG9" s="4" t="inlineStr"/>
+          <t>Approval B granted — awaiting owner review of docs PR</t>
+        </is>
+      </c>
+      <c r="AG9" s="4" t="inlineStr">
+        <is>
+          <t>Drafted 29 Oct 2026: docs/architecture/adr/ADR-001…018</t>
+        </is>
+      </c>
       <c r="AH9" s="4" t="inlineStr">
         <is>
           <t>None</t>
@@ -41409,7 +42746,7 @@
       </c>
       <c r="N21" s="4" t="inlineStr">
         <is>
-          <t>LS-001, LS-008</t>
+          <t>LS-001, LS-008, LS-009, LS-039</t>
         </is>
       </c>
       <c r="O21" s="4" t="inlineStr">
@@ -41536,7 +42873,7 @@
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>Create modules per ADR-002 (app, core:designsystem, core:ui, core:common, core:localization?, domain, data, feature:*) and convention plugins for shared config.</t>
+          <t>Create the 14 modules proposed in ADR-002 (:app, build-logic, :core:designsystem, :core:ui, :core:common, :domain, :data, :feature:onboarding/home/discover/create/reader/library/settings) and convention plugins for shared Android/Compose/test config.</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
@@ -45513,7 +46850,7 @@
       </c>
       <c r="K45" s="4" t="inlineStr">
         <is>
-          <t>:feature:profiles</t>
+          <t>:feature:settings</t>
         </is>
       </c>
       <c r="L45" s="5" t="inlineStr">
@@ -46373,7 +47710,7 @@
       </c>
       <c r="K50" s="4" t="inlineStr">
         <is>
-          <t>:feature:storydetails</t>
+          <t>:feature:discover</t>
         </is>
       </c>
       <c r="L50" s="5" t="inlineStr">
@@ -47923,7 +49260,7 @@
       </c>
       <c r="K59" s="4" t="inlineStr">
         <is>
-          <t>:feature:player</t>
+          <t>:feature:reader</t>
         </is>
       </c>
       <c r="L59" s="5" t="inlineStr">
@@ -48095,7 +49432,7 @@
       </c>
       <c r="K60" s="4" t="inlineStr">
         <is>
-          <t>:feature:player</t>
+          <t>:feature:reader</t>
         </is>
       </c>
       <c r="L60" s="5" t="inlineStr">
@@ -48266,7 +49603,7 @@
       </c>
       <c r="K61" s="4" t="inlineStr">
         <is>
-          <t>:feature:player</t>
+          <t>:feature:reader</t>
         </is>
       </c>
       <c r="L61" s="5" t="inlineStr">
@@ -49124,7 +50461,7 @@
       </c>
       <c r="K66" s="4" t="inlineStr">
         <is>
-          <t>:feature:notifications</t>
+          <t>:feature:settings</t>
         </is>
       </c>
       <c r="L66" s="5" t="inlineStr">
@@ -49295,7 +50632,7 @@
       </c>
       <c r="K67" s="4" t="inlineStr">
         <is>
-          <t>:feature:subscription</t>
+          <t>:feature:settings</t>
         </is>
       </c>
       <c r="L67" s="5" t="inlineStr">
@@ -51256,14 +52593,14 @@
       </c>
       <c r="AA78" s="4" t="inlineStr">
         <is>
-          <t>feature/LS-131-branch-strategy-pr-template-codeowners</t>
+          <t>claude/project-thread-veobz7</t>
         </is>
       </c>
       <c r="AB78" s="4" t="inlineStr"/>
       <c r="AC78" s="4" t="inlineStr"/>
       <c r="AD78" s="4" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>In Review</t>
         </is>
       </c>
       <c r="AE78" s="4" t="inlineStr">
@@ -51273,10 +52610,14 @@
       </c>
       <c r="AF78" s="4" t="inlineStr">
         <is>
-          <t>Awaiting Approval B</t>
-        </is>
-      </c>
-      <c r="AG78" s="4" t="inlineStr"/>
+          <t>Approval B granted — awaiting owner review of docs PR</t>
+        </is>
+      </c>
+      <c r="AG78" s="4" t="inlineStr">
+        <is>
+          <t>Drafted 29 Oct 2026: .github/pull_request_template.md, .github/CODEOWNERS (development branch awaits owner, D2)</t>
+        </is>
+      </c>
       <c r="AH78" s="4" t="inlineStr">
         <is>
           <t>None</t>
@@ -52091,14 +53432,14 @@
       </c>
       <c r="AA83" s="4" t="inlineStr">
         <is>
-          <t>feature/LS-150-configuration-docs-how-to-change</t>
+          <t>claude/project-thread-veobz7</t>
         </is>
       </c>
       <c r="AB83" s="4" t="inlineStr"/>
       <c r="AC83" s="4" t="inlineStr"/>
       <c r="AD83" s="4" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>In Review</t>
         </is>
       </c>
       <c r="AE83" s="4" t="inlineStr">
@@ -52108,10 +53449,14 @@
       </c>
       <c r="AF83" s="4" t="inlineStr">
         <is>
-          <t>Awaiting Approval B</t>
-        </is>
-      </c>
-      <c r="AG83" s="4" t="inlineStr"/>
+          <t>Approval B granted — awaiting owner review of docs PR</t>
+        </is>
+      </c>
+      <c r="AG83" s="4" t="inlineStr">
+        <is>
+          <t>Drafted 29 Oct 2026: docs/architecture/configuration-and-constants.md, how-to-change.md (drafted early in P1)</t>
+        </is>
+      </c>
       <c r="AH83" s="4" t="inlineStr">
         <is>
           <t>None</t>
@@ -52133,8 +53478,343 @@
         <v/>
       </c>
     </row>
+    <row r="84" ht="85" customHeight="1">
+      <c r="A84" s="17" t="inlineStr">
+        <is>
+          <t>LS-009</t>
+        </is>
+      </c>
+      <c r="B84" s="4" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C84" s="4" t="inlineStr">
+        <is>
+          <t>LS-EPIC-12</t>
+        </is>
+      </c>
+      <c r="D84" s="4" t="inlineStr">
+        <is>
+          <t>Repository hygiene: default branch main, development branch</t>
+        </is>
+      </c>
+      <c r="E84" s="4" t="inlineStr">
+        <is>
+          <t>Owner merges PR #1, sets the GitHub default branch back to main and creates development from main (decision D2, R-22).</t>
+        </is>
+      </c>
+      <c r="F84" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G84" s="4" t="inlineStr">
+        <is>
+          <t>Every branch and PR starts from the right base</t>
+        </is>
+      </c>
+      <c r="H84" s="4" t="inlineStr">
+        <is>
+          <t>Highest</t>
+        </is>
+      </c>
+      <c r="I84" s="4" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="J84" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K84" s="4" t="inlineStr">
+        <is>
+          <t>GitHub settings</t>
+        </is>
+      </c>
+      <c r="L84" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="M84" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N84" s="4" t="inlineStr">
+        <is>
+          <t>LS-001</t>
+        </is>
+      </c>
+      <c r="O84" s="4" t="inlineStr">
+        <is>
+          <t>Blocks: LS-030, LS-131
+Blocked by: LS-001</t>
+        </is>
+      </c>
+      <c r="P84" s="4" t="inlineStr">
+        <is>
+          <t>1. Default branch is main
+2. development exists from main
+3. PR #1 merged by owner</t>
+        </is>
+      </c>
+      <c r="Q84" s="4" t="inlineStr">
+        <is>
+          <t>Owner confirms settings changed</t>
+        </is>
+      </c>
+      <c r="R84" s="4" t="inlineStr">
+        <is>
+          <t>Owner action in GitHub settings; agents must not change repository settings.</t>
+        </is>
+      </c>
+      <c r="S84" s="4" t="inlineStr">
+        <is>
+          <t>Verify via GitHub API</t>
+        </is>
+      </c>
+      <c r="T84" s="4" t="n"/>
+      <c r="U84" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="V84" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="W84" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="X84" s="4" t="inlineStr">
+        <is>
+          <t>Release and Deployment Coordinator</t>
+        </is>
+      </c>
+      <c r="Y84" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z84" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="AA84" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="AB84" s="4" t="n"/>
+      <c r="AC84" s="4" t="n"/>
+      <c r="AD84" s="4" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="AE84" s="4" t="inlineStr">
+        <is>
+          <t>Project owner (human)</t>
+        </is>
+      </c>
+      <c r="AF84" s="4" t="inlineStr">
+        <is>
+          <t>Awaiting owner (D2)</t>
+        </is>
+      </c>
+      <c r="AG84" s="4" t="n"/>
+      <c r="AH84" s="4" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AI84" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AJ84" s="4" t="n"/>
+      <c r="AK84" s="4" t="n"/>
+      <c r="AL84" s="22">
+        <f>AD84&amp;"|"&amp;COUNTIF(AD$2:AD84,AD84)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="85" ht="85" customHeight="1">
+      <c r="A85" s="17" t="inlineStr">
+        <is>
+          <t>LS-039</t>
+        </is>
+      </c>
+      <c r="B85" s="4" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C85" s="4" t="inlineStr">
+        <is>
+          <t>LS-EPIC-12</t>
+        </is>
+      </c>
+      <c r="D85" s="4" t="inlineStr">
+        <is>
+          <t>Build verification environment (ADR-017)</t>
+        </is>
+      </c>
+      <c r="E85" s="4" t="inlineStr">
+        <is>
+          <t>Make Android builds verifiable for agent PRs: allow dl.google.com in the cloud environment network settings and rely on GitHub Actions (LS-130) as the shared runner (decision D3, R-21).</t>
+        </is>
+      </c>
+      <c r="F85" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G85" s="4" t="inlineStr">
+        <is>
+          <t>PRs carry real build and test evidence</t>
+        </is>
+      </c>
+      <c r="H85" s="4" t="inlineStr">
+        <is>
+          <t>Highest</t>
+        </is>
+      </c>
+      <c r="I85" s="4" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="J85" s="4" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="K85" s="4" t="inlineStr">
+        <is>
+          <t>Environment / CI</t>
+        </is>
+      </c>
+      <c r="L85" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="M85" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N85" s="4" t="inlineStr">
+        <is>
+          <t>LS-009</t>
+        </is>
+      </c>
+      <c r="O85" s="4" t="inlineStr">
+        <is>
+          <t>Blocks: LS-030, LS-035, LS-130
+Blocked by: LS-009</t>
+        </is>
+      </c>
+      <c r="P85" s="4" t="inlineStr">
+        <is>
+          <t>1. A Gradle sync that downloads AGP succeeds in the agent workspace or CI
+2. Decision recorded in ADR-017</t>
+        </is>
+      </c>
+      <c r="Q85" s="4" t="inlineStr">
+        <is>
+          <t>ADR-017 approved and verified with a real sync</t>
+        </is>
+      </c>
+      <c r="R85" s="4" t="inlineStr">
+        <is>
+          <t>Owner changes Network access in the project cloud environment; no credentials in the repo.</t>
+        </is>
+      </c>
+      <c r="S85" s="4" t="inlineStr">
+        <is>
+          <t>Gradle sync / assembleDebug run</t>
+        </is>
+      </c>
+      <c r="T85" s="4" t="n"/>
+      <c r="U85" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="V85" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="W85" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="X85" s="4" t="inlineStr">
+        <is>
+          <t>Build, Gradle &amp; CI/CD Engineer</t>
+        </is>
+      </c>
+      <c r="Y85" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z85" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="AA85" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="AB85" s="4" t="n"/>
+      <c r="AC85" s="4" t="n"/>
+      <c r="AD85" s="4" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="AE85" s="4" t="inlineStr">
+        <is>
+          <t>Project owner (human)</t>
+        </is>
+      </c>
+      <c r="AF85" s="4" t="inlineStr">
+        <is>
+          <t>Awaiting owner (D3)</t>
+        </is>
+      </c>
+      <c r="AG85" s="4" t="n"/>
+      <c r="AH85" s="4" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AI85" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AJ85" s="4" t="n"/>
+      <c r="AK85" s="4" t="n"/>
+      <c r="AL85" s="22">
+        <f>AD85&amp;"|"&amp;COUNTIF(AD$2:AD85,AD85)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AL83"/>
+  <autoFilter ref="A1:AL85"/>
   <conditionalFormatting sqref="AD2:AD83">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="5">
       <formula>"To Do"</formula>

</xml_diff>